<commit_message>
band-advance: rename Set Time -> Set Length; include it in the advance email
Set Length column (duration of the act's set; key kept as set_time internally).
Shows in the advance email ('Set length: 60 min' — numeric values get 'min') and
the status sheet. Template regenerated (35 cols) with the row preserved.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Code/BandInfoForm/tools/lists/advance_list_template.xlsx
+++ b/Code/BandInfoForm/tools/lists/advance_list_template.xlsx
@@ -636,7 +636,7 @@
       </c>
       <c r="Q2" s="4" t="inlineStr">
         <is>
-          <t>Set Time</t>
+          <t>Set Length</t>
         </is>
       </c>
       <c r="R2" s="4" t="inlineStr">
@@ -731,41 +731,113 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="5" t="n"/>
-      <c r="B3" s="5" t="n"/>
-      <c r="C3" s="5" t="n"/>
-      <c r="D3" s="5" t="n"/>
-      <c r="E3" s="5" t="n"/>
-      <c r="F3" s="5" t="n"/>
-      <c r="G3" s="5" t="n"/>
-      <c r="H3" s="5" t="n"/>
-      <c r="I3" s="5" t="n"/>
-      <c r="J3" s="5" t="n"/>
-      <c r="K3" s="5" t="n"/>
-      <c r="L3" s="5" t="n"/>
-      <c r="M3" s="5" t="n"/>
-      <c r="N3" s="5" t="n"/>
-      <c r="O3" s="5" t="n"/>
-      <c r="P3" s="5" t="n"/>
-      <c r="Q3" s="5" t="n"/>
-      <c r="R3" s="5" t="n"/>
-      <c r="S3" s="5" t="n"/>
-      <c r="T3" s="5" t="n"/>
-      <c r="U3" s="5" t="n"/>
-      <c r="V3" s="5" t="n"/>
-      <c r="W3" s="5" t="n"/>
-      <c r="X3" s="5" t="n"/>
-      <c r="Y3" s="5" t="n"/>
-      <c r="Z3" s="5" t="n"/>
-      <c r="AA3" s="5" t="n"/>
-      <c r="AB3" s="5" t="n"/>
-      <c r="AC3" s="5" t="n"/>
-      <c r="AD3" s="5" t="n"/>
-      <c r="AE3" s="5" t="n"/>
-      <c r="AF3" s="5" t="n"/>
-      <c r="AG3" s="5" t="n"/>
-      <c r="AH3" s="5" t="n"/>
-      <c r="AI3" s="5" t="n"/>
+      <c r="A3" s="5" t="inlineStr">
+        <is>
+          <t>513 Airwaves w/ Inhailer Radio</t>
+        </is>
+      </c>
+      <c r="B3" s="5" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="C3" s="5" t="inlineStr">
+        <is>
+          <t>Fountain Square</t>
+        </is>
+      </c>
+      <c r="D3" s="5" t="inlineStr">
+        <is>
+          <t>513 Airwaves w/ Inhailer Radio</t>
+        </is>
+      </c>
+      <c r="E3" s="5" t="inlineStr">
+        <is>
+          <t>Internal</t>
+        </is>
+      </c>
+      <c r="F3" s="5" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G3" s="5" t="inlineStr">
+        <is>
+          <t>INHAILER RADIO</t>
+        </is>
+      </c>
+      <c r="H3" s="5" t="inlineStr"/>
+      <c r="I3" s="5" t="inlineStr">
+        <is>
+          <t>Sam</t>
+        </is>
+      </c>
+      <c r="J3" s="5" t="inlineStr">
+        <is>
+          <t>5136214400</t>
+        </is>
+      </c>
+      <c r="K3" s="5" t="inlineStr">
+        <is>
+          <t>4:30pm</t>
+        </is>
+      </c>
+      <c r="L3" s="5" t="inlineStr">
+        <is>
+          <t>5:00pm</t>
+        </is>
+      </c>
+      <c r="M3" s="5" t="inlineStr">
+        <is>
+          <t>9pm</t>
+        </is>
+      </c>
+      <c r="N3" s="5" t="inlineStr">
+        <is>
+          <t>10pm</t>
+        </is>
+      </c>
+      <c r="O3" s="5" t="inlineStr">
+        <is>
+          <t>11pm</t>
+        </is>
+      </c>
+      <c r="P3" s="5" t="inlineStr">
+        <is>
+          <t>headliner</t>
+        </is>
+      </c>
+      <c r="Q3" s="5" t="inlineStr">
+        <is>
+          <t>60</t>
+        </is>
+      </c>
+      <c r="R3" s="5" t="inlineStr">
+        <is>
+          <t>Headiner Band</t>
+        </is>
+      </c>
+      <c r="S3" s="5" t="inlineStr">
+        <is>
+          <t>blloyd@3cdc.org</t>
+        </is>
+      </c>
+      <c r="T3" s="5" t="inlineStr"/>
+      <c r="U3" s="5" t="inlineStr"/>
+      <c r="V3" s="5" t="inlineStr"/>
+      <c r="W3" s="5" t="inlineStr"/>
+      <c r="X3" s="5" t="inlineStr"/>
+      <c r="Y3" s="5" t="inlineStr"/>
+      <c r="Z3" s="5" t="inlineStr"/>
+      <c r="AA3" s="5" t="inlineStr"/>
+      <c r="AB3" s="5" t="inlineStr"/>
+      <c r="AC3" s="5" t="inlineStr"/>
+      <c r="AD3" s="5" t="inlineStr"/>
+      <c r="AE3" s="5" t="inlineStr"/>
+      <c r="AF3" s="5" t="inlineStr"/>
+      <c r="AG3" s="5" t="inlineStr"/>
+      <c r="AH3" s="5" t="inlineStr"/>
+      <c r="AI3" s="5" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="6" t="n"/>
@@ -8406,7 +8478,7 @@
     <row r="13">
       <c r="A13" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">  ACT — slot, set time, the exact artist name, and the email the advance goes to.</t>
+          <t xml:space="preserve">  ACT — slot, set length, the exact artist name, and the email the advance goes to.</t>
         </is>
       </c>
     </row>

</xml_diff>